<commit_message>
Fix a pre-existing column-shift bug on Multimedia's External File in Forms row
Found while investigating the same class of bug just fixed for MM2: this
row's Automated?/Flow File values were shifted one column right (a
Maestro-Automatability-column value "Automatable" sitting in the
Automated? column), predating this session - the underlying automation
itself (scripts/run_appium_multimedia_suite.py --scenario
external_file_in_forms) is real and has been passing in CI every run
verified this session, just misfiled in the sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/[Master] Mobile Plan (2026).xlsx
+++ b/docs/[Master] Mobile Plan (2026).xlsx
@@ -11386,19 +11386,15 @@
       </c>
       <c r="I62" s="708" t="inlineStr">
         <is>
-          <t>Automatable</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J62" s="311" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K62" s="311" t="inlineStr">
-        <is>
           <t>scripts/run_appium_multimedia_suite.py --scenario external_file_in_forms (flows/multimedia/external_file_in_forms.yaml kept for reference, tagged superseded_by_appium)</t>
         </is>
       </c>
+      <c r="K62" s="311" t="n"/>
       <c r="L62" s="311" t="n"/>
       <c r="M62" s="311" t="n"/>
       <c r="N62" s="311" t="n"/>

</xml_diff>

<commit_message>
Confirm Form Submissions > Geoservice 1 (row 46) stays Not automatable
Investigated in depth rather than re-asserting the existing gap: the
Default Map Tileset property is reachable via a real HQ endpoint, but
which tileset is actually active has no observable signal anywhere on
device (confirmed via commcare-android source - GeoPointMapActivity/
EntityMapActivity call GoogleMap.setMapType() with nothing exposing
the active layer, and the SharedPreferences key that holds it is
unreadable since adb_shell is disabled on this BrowserStack tier).
Doing the row's own 3x publish/install/uninstall cycle against the
most shared app in this repo isn't worth it for a check with no
reliable pass/fail signal - same category as this tab's own Case
Lists 1/2 precedent. No HQ state was modified; investigation was
read-only throughout.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/[Master] Mobile Plan (2026).xlsx
+++ b/docs/[Master] Mobile Plan (2026).xlsx
@@ -14742,7 +14742,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="0" t="inlineStr">
         <is>
           <t>scripts/appium_case_search_claim_scenarios.py, scripts/run_case_search_claim_suite.py</t>
         </is>
@@ -26035,7 +26035,7 @@
       <c r="D46" s="564" t="n"/>
       <c r="E46" s="477" t="inlineStr">
         <is>
-          <t>This property will not update for user for App Updates (we don’t want to change the user experience on maps on App Updates).</t>
+          <t>This property will not update for user for App Updates (we don’t want to change the user experience on maps on App Updates). UPDATE (2026-09-16), investigated in depth (not just re-asserted), same category as Case Filters' own Case Lists 1/2 device-dependent visual-confirmation precedent: the tileset IS writable via a real HQ endpoint (cc-maps-default-layer, a named CommCare Profile Setting under app.profile.properties - a new write path would be needed since hq_client.py's existing set_custom_properties() targets a different dict), but on-device, the SELECTED tileset has no accessibility-tree signal anywhere (confirmed via commcare-android source: GeoPointMapActivity/EntityMapActivity just call GoogleMap.setMapType() with no Log/content-desc/resource-id exposing the active layer), and the SharedPreferences key that holds it is unreadable on this harness (adb_shell is disabled on BrowserStack's managed Appium server). A real map view IS already reached (unasserted) by the existing Partial appearance_attributes_page_through_and_submit.yaml flow. Given the actual tileset check has no reliable observable signal, the 3x publish/install/uninstall cycle against Basic Tests (the most shared app in this repo) isn't worth the blast radius for zero incremental confidence. See coverage/coverage_matrix.csv's Geoservice 1 row for the full citation. Stays Not automatable.</t>
         </is>
       </c>
       <c r="F46" s="204" t="n"/>

</xml_diff>

<commit_message>
Fix Multimedia Image Resize 5/10/15/20: Not automatable -> Partial
These 4 rows were labeled "Not automatable" while Automated? read
"Yes" - a real hq_setup/multimedia/image_resize_*.json artifact
exists and runs (attempting the HQ-side Auto-Resize Images setting
change), even though full end-to-end verification that the setting
took effect isn't possible. That's partial automation, not none -
the mirror image of the earlier Partial+No inconsistency fix.
Confirmed via a full-workbook sweep this is the only place this
exact pattern (Not automatable + plain "Yes") occurs; Recovery
Measures was checked separately and found clean.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/[Master] Mobile Plan (2026).xlsx
+++ b/docs/[Master] Mobile Plan (2026).xlsx
@@ -8909,7 +8909,7 @@
       <c r="G19" s="60" t="n"/>
       <c r="H19" s="60" t="inlineStr">
         <is>
-          <t>Not automatable</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="I19" s="709" t="inlineStr">
@@ -9214,7 +9214,7 @@
       <c r="G24" s="60" t="n"/>
       <c r="H24" s="60" t="inlineStr">
         <is>
-          <t>Not automatable</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="I24" s="709" t="inlineStr">
@@ -9516,7 +9516,7 @@
       <c r="G29" s="60" t="n"/>
       <c r="H29" s="60" t="inlineStr">
         <is>
-          <t>Not automatable</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="I29" s="709" t="inlineStr">
@@ -9818,7 +9818,7 @@
       <c r="G34" s="60" t="n"/>
       <c r="H34" s="60" t="inlineStr">
         <is>
-          <t>Not automatable</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="I34" s="709" t="inlineStr">

</xml_diff>